<commit_message>
Auto: refresh raw URLs for DawSathaporn
</commit_message>
<xml_diff>
--- a/data/DawSathaporn_all_raw.xlsx
+++ b/data/DawSathaporn_all_raw.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E103"/>
+  <dimension ref="A1:E105"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -446,7 +446,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>BEROKTO</t>
+          <t>BERDESEM</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -464,23 +464,23 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>https://raw.githubusercontent.com/DawSathaporn/BEROKTO/main/.github/workflows/main.yml</t>
+          <t>https://raw.githubusercontent.com/DawSathaporn/BERDESEM/main/.github/workflows/main.yml</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>BEROKTO</t>
+          <t>BERDESEM</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>BR01OKTOBER2026</t>
+          <t>BS01DESEMBER2026</t>
         </is>
       </c>
       <c r="C3" t="n">
-        <v>889425</v>
+        <v>889426</v>
       </c>
       <c r="D3" t="inlineStr">
         <is>
@@ -489,23 +489,23 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>https://raw.githubusercontent.com/DawSathaporn/BEROKTO/main/BR01OKTOBER2026</t>
+          <t>https://raw.githubusercontent.com/DawSathaporn/BERDESEM/main/BS01DESEMBER2026</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>BEROKTO</t>
+          <t>BERDESEM</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>BR02OKTOBER2026</t>
+          <t>BS02DESEMBER2026</t>
         </is>
       </c>
       <c r="C4" t="n">
-        <v>889425</v>
+        <v>889426</v>
       </c>
       <c r="D4" t="inlineStr">
         <is>
@@ -514,23 +514,23 @@
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>https://raw.githubusercontent.com/DawSathaporn/BEROKTO/main/BR02OKTOBER2026</t>
+          <t>https://raw.githubusercontent.com/DawSathaporn/BERDESEM/main/BS02DESEMBER2026</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>BEROKTO</t>
+          <t>BERDESEM</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>BR03OKTOBER2026</t>
+          <t>BS03DESEMBER2026</t>
         </is>
       </c>
       <c r="C5" t="n">
-        <v>889425</v>
+        <v>889426</v>
       </c>
       <c r="D5" t="inlineStr">
         <is>
@@ -539,23 +539,23 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>https://raw.githubusercontent.com/DawSathaporn/BEROKTO/main/BR03OKTOBER2026</t>
+          <t>https://raw.githubusercontent.com/DawSathaporn/BERDESEM/main/BS03DESEMBER2026</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>BEROKTO</t>
+          <t>BERDESEM</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>BR04OKTOBER2026</t>
+          <t>BS04DESEMBER2026</t>
         </is>
       </c>
       <c r="C6" t="n">
-        <v>889425</v>
+        <v>889426</v>
       </c>
       <c r="D6" t="inlineStr">
         <is>
@@ -564,23 +564,23 @@
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>https://raw.githubusercontent.com/DawSathaporn/BEROKTO/main/BR04OKTOBER2026</t>
+          <t>https://raw.githubusercontent.com/DawSathaporn/BERDESEM/main/BS04DESEMBER2026</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>BEROKTO</t>
+          <t>BERDESEM</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>BR05OKTOBER2026</t>
+          <t>BS05DESEMBER2026</t>
         </is>
       </c>
       <c r="C7" t="n">
-        <v>889425</v>
+        <v>889426</v>
       </c>
       <c r="D7" t="inlineStr">
         <is>
@@ -589,23 +589,23 @@
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>https://raw.githubusercontent.com/DawSathaporn/BEROKTO/main/BR05OKTOBER2026</t>
+          <t>https://raw.githubusercontent.com/DawSathaporn/BERDESEM/main/BS05DESEMBER2026</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>BEROKTO</t>
+          <t>BERDESEM</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>BR06OKTOBER2026</t>
+          <t>BS06DESEMBER2026</t>
         </is>
       </c>
       <c r="C8" t="n">
-        <v>889425</v>
+        <v>889426</v>
       </c>
       <c r="D8" t="inlineStr">
         <is>
@@ -614,23 +614,23 @@
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>https://raw.githubusercontent.com/DawSathaporn/BEROKTO/main/BR06OKTOBER2026</t>
+          <t>https://raw.githubusercontent.com/DawSathaporn/BERDESEM/main/BS06DESEMBER2026</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>BEROKTO</t>
+          <t>BERDESEM</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>BR07OKTOBER2026</t>
+          <t>BS07DESEMBER2026</t>
         </is>
       </c>
       <c r="C9" t="n">
-        <v>889425</v>
+        <v>889426</v>
       </c>
       <c r="D9" t="inlineStr">
         <is>
@@ -639,23 +639,23 @@
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>https://raw.githubusercontent.com/DawSathaporn/BEROKTO/main/BR07OKTOBER2026</t>
+          <t>https://raw.githubusercontent.com/DawSathaporn/BERDESEM/main/BS07DESEMBER2026</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>BEROKTO</t>
+          <t>BERDESEM</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>BR08OKTOBER2026</t>
+          <t>BS08DESEMBER2026</t>
         </is>
       </c>
       <c r="C10" t="n">
-        <v>889425</v>
+        <v>889426</v>
       </c>
       <c r="D10" t="inlineStr">
         <is>
@@ -664,23 +664,23 @@
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>https://raw.githubusercontent.com/DawSathaporn/BEROKTO/main/BR08OKTOBER2026</t>
+          <t>https://raw.githubusercontent.com/DawSathaporn/BERDESEM/main/BS08DESEMBER2026</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>BEROKTO</t>
+          <t>BERDESEM</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>BR09OKTOBER2026</t>
+          <t>BS09DESEMBER2026</t>
         </is>
       </c>
       <c r="C11" t="n">
-        <v>889425</v>
+        <v>889426</v>
       </c>
       <c r="D11" t="inlineStr">
         <is>
@@ -689,23 +689,23 @@
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>https://raw.githubusercontent.com/DawSathaporn/BEROKTO/main/BR09OKTOBER2026</t>
+          <t>https://raw.githubusercontent.com/DawSathaporn/BERDESEM/main/BS09DESEMBER2026</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>BEROKTO</t>
+          <t>BERDESEM</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>BR10OKTOBER2026</t>
+          <t>BS10DESEMBER2026</t>
         </is>
       </c>
       <c r="C12" t="n">
-        <v>889425</v>
+        <v>889426</v>
       </c>
       <c r="D12" t="inlineStr">
         <is>
@@ -714,23 +714,23 @@
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>https://raw.githubusercontent.com/DawSathaporn/BEROKTO/main/BR10OKTOBER2026</t>
+          <t>https://raw.githubusercontent.com/DawSathaporn/BERDESEM/main/BS10DESEMBER2026</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>BEROKTO</t>
+          <t>BERDESEM</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>BR11OKTOBER2026</t>
+          <t>BS11DESEMBER2026</t>
         </is>
       </c>
       <c r="C13" t="n">
-        <v>889425</v>
+        <v>889426</v>
       </c>
       <c r="D13" t="inlineStr">
         <is>
@@ -739,23 +739,23 @@
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>https://raw.githubusercontent.com/DawSathaporn/BEROKTO/main/BR11OKTOBER2026</t>
+          <t>https://raw.githubusercontent.com/DawSathaporn/BERDESEM/main/BS11DESEMBER2026</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>BEROKTO</t>
+          <t>BERDESEM</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>BR12OKTOBER2026</t>
+          <t>BS12DESEMBER2026</t>
         </is>
       </c>
       <c r="C14" t="n">
-        <v>889425</v>
+        <v>889426</v>
       </c>
       <c r="D14" t="inlineStr">
         <is>
@@ -764,23 +764,23 @@
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>https://raw.githubusercontent.com/DawSathaporn/BEROKTO/main/BR12OKTOBER2026</t>
+          <t>https://raw.githubusercontent.com/DawSathaporn/BERDESEM/main/BS12DESEMBER2026</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>BEROKTO</t>
+          <t>BERDESEM</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>BR13OKTOBER2026</t>
+          <t>BS13DESEMBER2026</t>
         </is>
       </c>
       <c r="C15" t="n">
-        <v>889425</v>
+        <v>889426</v>
       </c>
       <c r="D15" t="inlineStr">
         <is>
@@ -789,23 +789,23 @@
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>https://raw.githubusercontent.com/DawSathaporn/BEROKTO/main/BR13OKTOBER2026</t>
+          <t>https://raw.githubusercontent.com/DawSathaporn/BERDESEM/main/BS13DESEMBER2026</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>BEROKTO</t>
+          <t>BERDESEM</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>BR14OKTOBER2026</t>
+          <t>BS14DESEMBER2026</t>
         </is>
       </c>
       <c r="C16" t="n">
-        <v>889425</v>
+        <v>889426</v>
       </c>
       <c r="D16" t="inlineStr">
         <is>
@@ -814,23 +814,23 @@
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>https://raw.githubusercontent.com/DawSathaporn/BEROKTO/main/BR14OKTOBER2026</t>
+          <t>https://raw.githubusercontent.com/DawSathaporn/BERDESEM/main/BS14DESEMBER2026</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>BEROKTO</t>
+          <t>BERDESEM</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>BR15OKTOBER2026</t>
+          <t>BS15DESEMBER2026</t>
         </is>
       </c>
       <c r="C17" t="n">
-        <v>889425</v>
+        <v>889426</v>
       </c>
       <c r="D17" t="inlineStr">
         <is>
@@ -839,23 +839,23 @@
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>https://raw.githubusercontent.com/DawSathaporn/BEROKTO/main/BR15OKTOBER2026</t>
+          <t>https://raw.githubusercontent.com/DawSathaporn/BERDESEM/main/BS15DESEMBER2026</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>BEROKTO</t>
+          <t>BERDESEM</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>BR16OKTOBER2026</t>
+          <t>BS16DESEMBER2026</t>
         </is>
       </c>
       <c r="C18" t="n">
-        <v>889425</v>
+        <v>889426</v>
       </c>
       <c r="D18" t="inlineStr">
         <is>
@@ -864,23 +864,23 @@
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>https://raw.githubusercontent.com/DawSathaporn/BEROKTO/main/BR16OKTOBER2026</t>
+          <t>https://raw.githubusercontent.com/DawSathaporn/BERDESEM/main/BS16DESEMBER2026</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>BEROKTO</t>
+          <t>BERDESEM</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>BR17OKTOBER2026</t>
+          <t>BS17DESEMBER2026</t>
         </is>
       </c>
       <c r="C19" t="n">
-        <v>889425</v>
+        <v>889426</v>
       </c>
       <c r="D19" t="inlineStr">
         <is>
@@ -889,23 +889,23 @@
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>https://raw.githubusercontent.com/DawSathaporn/BEROKTO/main/BR17OKTOBER2026</t>
+          <t>https://raw.githubusercontent.com/DawSathaporn/BERDESEM/main/BS17DESEMBER2026</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>BEROKTO</t>
+          <t>BERDESEM</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>BR18OKTOBER2026</t>
+          <t>BS18DESEMBER2026</t>
         </is>
       </c>
       <c r="C20" t="n">
-        <v>889425</v>
+        <v>889426</v>
       </c>
       <c r="D20" t="inlineStr">
         <is>
@@ -914,23 +914,23 @@
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>https://raw.githubusercontent.com/DawSathaporn/BEROKTO/main/BR18OKTOBER2026</t>
+          <t>https://raw.githubusercontent.com/DawSathaporn/BERDESEM/main/BS18DESEMBER2026</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>BEROKTO</t>
+          <t>BERDESEM</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>BR19OKTOBER2026</t>
+          <t>BS19DESEMBER2026</t>
         </is>
       </c>
       <c r="C21" t="n">
-        <v>889425</v>
+        <v>889426</v>
       </c>
       <c r="D21" t="inlineStr">
         <is>
@@ -939,23 +939,23 @@
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>https://raw.githubusercontent.com/DawSathaporn/BEROKTO/main/BR19OKTOBER2026</t>
+          <t>https://raw.githubusercontent.com/DawSathaporn/BERDESEM/main/BS19DESEMBER2026</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>BEROKTO</t>
+          <t>BERDESEM</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>BR20OKTOBER2026</t>
+          <t>BS20DESEMBER2026</t>
         </is>
       </c>
       <c r="C22" t="n">
-        <v>889425</v>
+        <v>889426</v>
       </c>
       <c r="D22" t="inlineStr">
         <is>
@@ -964,23 +964,23 @@
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>https://raw.githubusercontent.com/DawSathaporn/BEROKTO/main/BR20OKTOBER2026</t>
+          <t>https://raw.githubusercontent.com/DawSathaporn/BERDESEM/main/BS20DESEMBER2026</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>BEROKTO</t>
+          <t>BERDESEM</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>BR21OKTOBER2026</t>
+          <t>BS21DESEMBER2026</t>
         </is>
       </c>
       <c r="C23" t="n">
-        <v>889425</v>
+        <v>889426</v>
       </c>
       <c r="D23" t="inlineStr">
         <is>
@@ -989,23 +989,23 @@
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>https://raw.githubusercontent.com/DawSathaporn/BEROKTO/main/BR21OKTOBER2026</t>
+          <t>https://raw.githubusercontent.com/DawSathaporn/BERDESEM/main/BS21DESEMBER2026</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>BEROKTO</t>
+          <t>BERDESEM</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>BR22OKTOBER2026</t>
+          <t>BS22DESEMBER2026</t>
         </is>
       </c>
       <c r="C24" t="n">
-        <v>889425</v>
+        <v>889426</v>
       </c>
       <c r="D24" t="inlineStr">
         <is>
@@ -1014,23 +1014,23 @@
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>https://raw.githubusercontent.com/DawSathaporn/BEROKTO/main/BR22OKTOBER2026</t>
+          <t>https://raw.githubusercontent.com/DawSathaporn/BERDESEM/main/BS22DESEMBER2026</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>BEROKTO</t>
+          <t>BERDESEM</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>BR23OKTOBER2026</t>
+          <t>BS23DESEMBER2026</t>
         </is>
       </c>
       <c r="C25" t="n">
-        <v>889425</v>
+        <v>889426</v>
       </c>
       <c r="D25" t="inlineStr">
         <is>
@@ -1039,23 +1039,23 @@
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>https://raw.githubusercontent.com/DawSathaporn/BEROKTO/main/BR23OKTOBER2026</t>
+          <t>https://raw.githubusercontent.com/DawSathaporn/BERDESEM/main/BS23DESEMBER2026</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>BEROKTO</t>
+          <t>BERDESEM</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>BR24OKTOBER2026</t>
+          <t>BS24DESEMBER2026</t>
         </is>
       </c>
       <c r="C26" t="n">
-        <v>889425</v>
+        <v>889426</v>
       </c>
       <c r="D26" t="inlineStr">
         <is>
@@ -1064,23 +1064,23 @@
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>https://raw.githubusercontent.com/DawSathaporn/BEROKTO/main/BR24OKTOBER2026</t>
+          <t>https://raw.githubusercontent.com/DawSathaporn/BERDESEM/main/BS24DESEMBER2026</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>BEROKTO</t>
+          <t>BERDESEM</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>BR25OKTOBER2026</t>
+          <t>BS25DESEMBER2026</t>
         </is>
       </c>
       <c r="C27" t="n">
-        <v>889425</v>
+        <v>889426</v>
       </c>
       <c r="D27" t="inlineStr">
         <is>
@@ -1089,23 +1089,23 @@
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>https://raw.githubusercontent.com/DawSathaporn/BEROKTO/main/BR25OKTOBER2026</t>
+          <t>https://raw.githubusercontent.com/DawSathaporn/BERDESEM/main/BS25DESEMBER2026</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>BEROKTO</t>
+          <t>BERDESEM</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>BR26OKTOBER2026</t>
+          <t>BS26DESEMBER2026</t>
         </is>
       </c>
       <c r="C28" t="n">
-        <v>889425</v>
+        <v>889426</v>
       </c>
       <c r="D28" t="inlineStr">
         <is>
@@ -1114,23 +1114,23 @@
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>https://raw.githubusercontent.com/DawSathaporn/BEROKTO/main/BR26OKTOBER2026</t>
+          <t>https://raw.githubusercontent.com/DawSathaporn/BERDESEM/main/BS26DESEMBER2026</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>BEROKTO</t>
+          <t>BERDESEM</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>BR27OKTOBER2026</t>
+          <t>BS27DESEMBER2026</t>
         </is>
       </c>
       <c r="C29" t="n">
-        <v>889425</v>
+        <v>889426</v>
       </c>
       <c r="D29" t="inlineStr">
         <is>
@@ -1139,23 +1139,23 @@
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>https://raw.githubusercontent.com/DawSathaporn/BEROKTO/main/BR27OKTOBER2026</t>
+          <t>https://raw.githubusercontent.com/DawSathaporn/BERDESEM/main/BS27DESEMBER2026</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>BEROKTO</t>
+          <t>BERDESEM</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>BR28OKTOBER2026</t>
+          <t>BS28DESEMBER2026</t>
         </is>
       </c>
       <c r="C30" t="n">
-        <v>889425</v>
+        <v>889426</v>
       </c>
       <c r="D30" t="inlineStr">
         <is>
@@ -1164,23 +1164,23 @@
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>https://raw.githubusercontent.com/DawSathaporn/BEROKTO/main/BR28OKTOBER2026</t>
+          <t>https://raw.githubusercontent.com/DawSathaporn/BERDESEM/main/BS28DESEMBER2026</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>BEROKTO</t>
+          <t>BERDESEM</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>BR29OKTOBER2026</t>
+          <t>BS29DESEMBER2026</t>
         </is>
       </c>
       <c r="C31" t="n">
-        <v>889425</v>
+        <v>889426</v>
       </c>
       <c r="D31" t="inlineStr">
         <is>
@@ -1189,23 +1189,23 @@
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>https://raw.githubusercontent.com/DawSathaporn/BEROKTO/main/BR29OKTOBER2026</t>
+          <t>https://raw.githubusercontent.com/DawSathaporn/BERDESEM/main/BS29DESEMBER2026</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>BEROKTO</t>
+          <t>BERDESEM</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>BR30OKTOBER2026</t>
+          <t>BS30DESEMBER2026</t>
         </is>
       </c>
       <c r="C32" t="n">
-        <v>889425</v>
+        <v>889426</v>
       </c>
       <c r="D32" t="inlineStr">
         <is>
@@ -1214,23 +1214,23 @@
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>https://raw.githubusercontent.com/DawSathaporn/BEROKTO/main/BR30OKTOBER2026</t>
+          <t>https://raw.githubusercontent.com/DawSathaporn/BERDESEM/main/BS30DESEMBER2026</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>BEROKTO</t>
+          <t>BERDESEM</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>BR31OKTOBER2026</t>
+          <t>BS31DESEMBER2026</t>
         </is>
       </c>
       <c r="C33" t="n">
-        <v>889425</v>
+        <v>889426</v>
       </c>
       <c r="D33" t="inlineStr">
         <is>
@@ -1239,14 +1239,14 @@
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>https://raw.githubusercontent.com/DawSathaporn/BEROKTO/main/BR31OKTOBER2026</t>
+          <t>https://raw.githubusercontent.com/DawSathaporn/BERDESEM/main/BS31DESEMBER2026</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>BEROKTO</t>
+          <t>BERDESEM</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
@@ -1255,7 +1255,7 @@
         </is>
       </c>
       <c r="C34" t="n">
-        <v>15172</v>
+        <v>15175</v>
       </c>
       <c r="D34" t="inlineStr">
         <is>
@@ -1264,23 +1264,23 @@
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>https://raw.githubusercontent.com/DawSathaporn/BEROKTO/main/update_github_file.py</t>
+          <t>https://raw.githubusercontent.com/DawSathaporn/BERDESEM/main/update_github_file.py</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>UGR</t>
+          <t>BERNOVEM</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>.github/workflows/raw-urls.yml</t>
+          <t>.github/workflows/main.yml</t>
         </is>
       </c>
       <c r="C35" t="n">
-        <v>2174</v>
+        <v>851</v>
       </c>
       <c r="D35" t="inlineStr">
         <is>
@@ -1289,23 +1289,23 @@
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>https://raw.githubusercontent.com/DawSathaporn/UGR/main/.github/workflows/raw-urls.yml</t>
+          <t>https://raw.githubusercontent.com/DawSathaporn/BERNOVEM/main/.github/workflows/main.yml</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>UGR</t>
+          <t>BERNOVEM</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>data/uppermoon77_all_raw.csv</t>
+          <t>BN01NOVEMBER2026</t>
         </is>
       </c>
       <c r="C36" t="n">
-        <v>41907</v>
+        <v>889426</v>
       </c>
       <c r="D36" t="inlineStr">
         <is>
@@ -1314,23 +1314,23 @@
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>https://raw.githubusercontent.com/DawSathaporn/UGR/main/data/uppermoon77_all_raw.csv</t>
+          <t>https://raw.githubusercontent.com/DawSathaporn/BERNOVEM/main/BN01NOVEMBER2026</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>UGR</t>
+          <t>BERNOVEM</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>data/uppermoon77_all_raw.xlsx</t>
+          <t>BN02NOVEMBER2026</t>
         </is>
       </c>
       <c r="C37" t="n">
-        <v>15208</v>
+        <v>889426</v>
       </c>
       <c r="D37" t="inlineStr">
         <is>
@@ -1339,23 +1339,23 @@
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>https://raw.githubusercontent.com/DawSathaporn/UGR/main/data/uppermoon77_all_raw.xlsx</t>
+          <t>https://raw.githubusercontent.com/DawSathaporn/BERNOVEM/main/BN02NOVEMBER2026</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>UGR</t>
+          <t>BERNOVEM</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>generate_all_repos_raw_urls.py</t>
+          <t>BN03NOVEMBER2026</t>
         </is>
       </c>
       <c r="C38" t="n">
-        <v>6543</v>
+        <v>889426</v>
       </c>
       <c r="D38" t="inlineStr">
         <is>
@@ -1364,7 +1364,7 @@
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>https://raw.githubusercontent.com/DawSathaporn/UGR/main/generate_all_repos_raw_urls.py</t>
+          <t>https://raw.githubusercontent.com/DawSathaporn/BERNOVEM/main/BN03NOVEMBER2026</t>
         </is>
       </c>
     </row>
@@ -1376,11 +1376,11 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>.github/workflows/main.yml</t>
+          <t>BN04NOVEMBER2026</t>
         </is>
       </c>
       <c r="C39" t="n">
-        <v>851</v>
+        <v>889426</v>
       </c>
       <c r="D39" t="inlineStr">
         <is>
@@ -1389,7 +1389,7 @@
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>https://raw.githubusercontent.com/DawSathaporn/BERNOVEM/main/.github/workflows/main.yml</t>
+          <t>https://raw.githubusercontent.com/DawSathaporn/BERNOVEM/main/BN04NOVEMBER2026</t>
         </is>
       </c>
     </row>
@@ -1401,7 +1401,7 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>BN01NOVEMBER2026</t>
+          <t>BN05NOVEMBER2026</t>
         </is>
       </c>
       <c r="C40" t="n">
@@ -1414,7 +1414,7 @@
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>https://raw.githubusercontent.com/DawSathaporn/BERNOVEM/main/BN01NOVEMBER2026</t>
+          <t>https://raw.githubusercontent.com/DawSathaporn/BERNOVEM/main/BN05NOVEMBER2026</t>
         </is>
       </c>
     </row>
@@ -1426,7 +1426,7 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>BN02NOVEMBER2026</t>
+          <t>BN06NOVEMBER2026</t>
         </is>
       </c>
       <c r="C41" t="n">
@@ -1439,7 +1439,7 @@
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>https://raw.githubusercontent.com/DawSathaporn/BERNOVEM/main/BN02NOVEMBER2026</t>
+          <t>https://raw.githubusercontent.com/DawSathaporn/BERNOVEM/main/BN06NOVEMBER2026</t>
         </is>
       </c>
     </row>
@@ -1451,7 +1451,7 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>BN03NOVEMBER2026</t>
+          <t>BN07NOVEMBER2026</t>
         </is>
       </c>
       <c r="C42" t="n">
@@ -1464,7 +1464,7 @@
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>https://raw.githubusercontent.com/DawSathaporn/BERNOVEM/main/BN03NOVEMBER2026</t>
+          <t>https://raw.githubusercontent.com/DawSathaporn/BERNOVEM/main/BN07NOVEMBER2026</t>
         </is>
       </c>
     </row>
@@ -1476,7 +1476,7 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>BN04NOVEMBER2026</t>
+          <t>BN08NOVEMBER2026</t>
         </is>
       </c>
       <c r="C43" t="n">
@@ -1489,7 +1489,7 @@
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>https://raw.githubusercontent.com/DawSathaporn/BERNOVEM/main/BN04NOVEMBER2026</t>
+          <t>https://raw.githubusercontent.com/DawSathaporn/BERNOVEM/main/BN08NOVEMBER2026</t>
         </is>
       </c>
     </row>
@@ -1501,7 +1501,7 @@
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>BN05NOVEMBER2026</t>
+          <t>BN09NOVEMBER2026</t>
         </is>
       </c>
       <c r="C44" t="n">
@@ -1514,7 +1514,7 @@
       </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t>https://raw.githubusercontent.com/DawSathaporn/BERNOVEM/main/BN05NOVEMBER2026</t>
+          <t>https://raw.githubusercontent.com/DawSathaporn/BERNOVEM/main/BN09NOVEMBER2026</t>
         </is>
       </c>
     </row>
@@ -1526,7 +1526,7 @@
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>BN06NOVEMBER2026</t>
+          <t>BN10NOVEMBER2026</t>
         </is>
       </c>
       <c r="C45" t="n">
@@ -1539,7 +1539,7 @@
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>https://raw.githubusercontent.com/DawSathaporn/BERNOVEM/main/BN06NOVEMBER2026</t>
+          <t>https://raw.githubusercontent.com/DawSathaporn/BERNOVEM/main/BN10NOVEMBER2026</t>
         </is>
       </c>
     </row>
@@ -1551,7 +1551,7 @@
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>BN07NOVEMBER2026</t>
+          <t>BN11NOVEMBER2026</t>
         </is>
       </c>
       <c r="C46" t="n">
@@ -1564,7 +1564,7 @@
       </c>
       <c r="E46" t="inlineStr">
         <is>
-          <t>https://raw.githubusercontent.com/DawSathaporn/BERNOVEM/main/BN07NOVEMBER2026</t>
+          <t>https://raw.githubusercontent.com/DawSathaporn/BERNOVEM/main/BN11NOVEMBER2026</t>
         </is>
       </c>
     </row>
@@ -1576,7 +1576,7 @@
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>BN08NOVEMBER2026</t>
+          <t>BN12NOVEMBER2026</t>
         </is>
       </c>
       <c r="C47" t="n">
@@ -1589,7 +1589,7 @@
       </c>
       <c r="E47" t="inlineStr">
         <is>
-          <t>https://raw.githubusercontent.com/DawSathaporn/BERNOVEM/main/BN08NOVEMBER2026</t>
+          <t>https://raw.githubusercontent.com/DawSathaporn/BERNOVEM/main/BN12NOVEMBER2026</t>
         </is>
       </c>
     </row>
@@ -1601,7 +1601,7 @@
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>BN09NOVEMBER2026</t>
+          <t>BN13NOVEMBER2026</t>
         </is>
       </c>
       <c r="C48" t="n">
@@ -1614,7 +1614,7 @@
       </c>
       <c r="E48" t="inlineStr">
         <is>
-          <t>https://raw.githubusercontent.com/DawSathaporn/BERNOVEM/main/BN09NOVEMBER2026</t>
+          <t>https://raw.githubusercontent.com/DawSathaporn/BERNOVEM/main/BN13NOVEMBER2026</t>
         </is>
       </c>
     </row>
@@ -1626,7 +1626,7 @@
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>BN10NOVEMBER2026</t>
+          <t>BN14NOVEMBER2026</t>
         </is>
       </c>
       <c r="C49" t="n">
@@ -1639,7 +1639,7 @@
       </c>
       <c r="E49" t="inlineStr">
         <is>
-          <t>https://raw.githubusercontent.com/DawSathaporn/BERNOVEM/main/BN10NOVEMBER2026</t>
+          <t>https://raw.githubusercontent.com/DawSathaporn/BERNOVEM/main/BN14NOVEMBER2026</t>
         </is>
       </c>
     </row>
@@ -1651,7 +1651,7 @@
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>BN11NOVEMBER2026</t>
+          <t>BN15NOVEMBER2026</t>
         </is>
       </c>
       <c r="C50" t="n">
@@ -1664,7 +1664,7 @@
       </c>
       <c r="E50" t="inlineStr">
         <is>
-          <t>https://raw.githubusercontent.com/DawSathaporn/BERNOVEM/main/BN11NOVEMBER2026</t>
+          <t>https://raw.githubusercontent.com/DawSathaporn/BERNOVEM/main/BN15NOVEMBER2026</t>
         </is>
       </c>
     </row>
@@ -1676,7 +1676,7 @@
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>BN12NOVEMBER2026</t>
+          <t>BN16NOVEMBER2026</t>
         </is>
       </c>
       <c r="C51" t="n">
@@ -1689,7 +1689,7 @@
       </c>
       <c r="E51" t="inlineStr">
         <is>
-          <t>https://raw.githubusercontent.com/DawSathaporn/BERNOVEM/main/BN12NOVEMBER2026</t>
+          <t>https://raw.githubusercontent.com/DawSathaporn/BERNOVEM/main/BN16NOVEMBER2026</t>
         </is>
       </c>
     </row>
@@ -1701,7 +1701,7 @@
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>BN13NOVEMBER2026</t>
+          <t>BN17NOVEMBER2026</t>
         </is>
       </c>
       <c r="C52" t="n">
@@ -1714,7 +1714,7 @@
       </c>
       <c r="E52" t="inlineStr">
         <is>
-          <t>https://raw.githubusercontent.com/DawSathaporn/BERNOVEM/main/BN13NOVEMBER2026</t>
+          <t>https://raw.githubusercontent.com/DawSathaporn/BERNOVEM/main/BN17NOVEMBER2026</t>
         </is>
       </c>
     </row>
@@ -1726,7 +1726,7 @@
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>BN14NOVEMBER2026</t>
+          <t>BN18NOVEMBER2026</t>
         </is>
       </c>
       <c r="C53" t="n">
@@ -1739,7 +1739,7 @@
       </c>
       <c r="E53" t="inlineStr">
         <is>
-          <t>https://raw.githubusercontent.com/DawSathaporn/BERNOVEM/main/BN14NOVEMBER2026</t>
+          <t>https://raw.githubusercontent.com/DawSathaporn/BERNOVEM/main/BN18NOVEMBER2026</t>
         </is>
       </c>
     </row>
@@ -1751,7 +1751,7 @@
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>BN15NOVEMBER2026</t>
+          <t>BN19NOVEMBER2026</t>
         </is>
       </c>
       <c r="C54" t="n">
@@ -1764,7 +1764,7 @@
       </c>
       <c r="E54" t="inlineStr">
         <is>
-          <t>https://raw.githubusercontent.com/DawSathaporn/BERNOVEM/main/BN15NOVEMBER2026</t>
+          <t>https://raw.githubusercontent.com/DawSathaporn/BERNOVEM/main/BN19NOVEMBER2026</t>
         </is>
       </c>
     </row>
@@ -1776,7 +1776,7 @@
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>BN16NOVEMBER2026</t>
+          <t>BN20NOVEMBER2026</t>
         </is>
       </c>
       <c r="C55" t="n">
@@ -1789,7 +1789,7 @@
       </c>
       <c r="E55" t="inlineStr">
         <is>
-          <t>https://raw.githubusercontent.com/DawSathaporn/BERNOVEM/main/BN16NOVEMBER2026</t>
+          <t>https://raw.githubusercontent.com/DawSathaporn/BERNOVEM/main/BN20NOVEMBER2026</t>
         </is>
       </c>
     </row>
@@ -1801,7 +1801,7 @@
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>BN17NOVEMBER2026</t>
+          <t>BN21NOVEMBER2026</t>
         </is>
       </c>
       <c r="C56" t="n">
@@ -1814,7 +1814,7 @@
       </c>
       <c r="E56" t="inlineStr">
         <is>
-          <t>https://raw.githubusercontent.com/DawSathaporn/BERNOVEM/main/BN17NOVEMBER2026</t>
+          <t>https://raw.githubusercontent.com/DawSathaporn/BERNOVEM/main/BN21NOVEMBER2026</t>
         </is>
       </c>
     </row>
@@ -1826,7 +1826,7 @@
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>BN18NOVEMBER2026</t>
+          <t>BN22NOVEMBER2026</t>
         </is>
       </c>
       <c r="C57" t="n">
@@ -1839,7 +1839,7 @@
       </c>
       <c r="E57" t="inlineStr">
         <is>
-          <t>https://raw.githubusercontent.com/DawSathaporn/BERNOVEM/main/BN18NOVEMBER2026</t>
+          <t>https://raw.githubusercontent.com/DawSathaporn/BERNOVEM/main/BN22NOVEMBER2026</t>
         </is>
       </c>
     </row>
@@ -1851,7 +1851,7 @@
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>BN19NOVEMBER2026</t>
+          <t>BN23NOVEMBER2026</t>
         </is>
       </c>
       <c r="C58" t="n">
@@ -1864,7 +1864,7 @@
       </c>
       <c r="E58" t="inlineStr">
         <is>
-          <t>https://raw.githubusercontent.com/DawSathaporn/BERNOVEM/main/BN19NOVEMBER2026</t>
+          <t>https://raw.githubusercontent.com/DawSathaporn/BERNOVEM/main/BN23NOVEMBER2026</t>
         </is>
       </c>
     </row>
@@ -1876,7 +1876,7 @@
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>BN20NOVEMBER2026</t>
+          <t>BN24NOVEMBER2026</t>
         </is>
       </c>
       <c r="C59" t="n">
@@ -1889,7 +1889,7 @@
       </c>
       <c r="E59" t="inlineStr">
         <is>
-          <t>https://raw.githubusercontent.com/DawSathaporn/BERNOVEM/main/BN20NOVEMBER2026</t>
+          <t>https://raw.githubusercontent.com/DawSathaporn/BERNOVEM/main/BN24NOVEMBER2026</t>
         </is>
       </c>
     </row>
@@ -1901,7 +1901,7 @@
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>BN21NOVEMBER2026</t>
+          <t>BN25NOVEMBER2026</t>
         </is>
       </c>
       <c r="C60" t="n">
@@ -1914,7 +1914,7 @@
       </c>
       <c r="E60" t="inlineStr">
         <is>
-          <t>https://raw.githubusercontent.com/DawSathaporn/BERNOVEM/main/BN21NOVEMBER2026</t>
+          <t>https://raw.githubusercontent.com/DawSathaporn/BERNOVEM/main/BN25NOVEMBER2026</t>
         </is>
       </c>
     </row>
@@ -1926,7 +1926,7 @@
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>BN22NOVEMBER2026</t>
+          <t>BN26NOVEMBER2026</t>
         </is>
       </c>
       <c r="C61" t="n">
@@ -1939,7 +1939,7 @@
       </c>
       <c r="E61" t="inlineStr">
         <is>
-          <t>https://raw.githubusercontent.com/DawSathaporn/BERNOVEM/main/BN22NOVEMBER2026</t>
+          <t>https://raw.githubusercontent.com/DawSathaporn/BERNOVEM/main/BN26NOVEMBER2026</t>
         </is>
       </c>
     </row>
@@ -1951,7 +1951,7 @@
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>BN23NOVEMBER2026</t>
+          <t>BN27NOVEMBER2026</t>
         </is>
       </c>
       <c r="C62" t="n">
@@ -1964,7 +1964,7 @@
       </c>
       <c r="E62" t="inlineStr">
         <is>
-          <t>https://raw.githubusercontent.com/DawSathaporn/BERNOVEM/main/BN23NOVEMBER2026</t>
+          <t>https://raw.githubusercontent.com/DawSathaporn/BERNOVEM/main/BN27NOVEMBER2026</t>
         </is>
       </c>
     </row>
@@ -1976,7 +1976,7 @@
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>BN24NOVEMBER2026</t>
+          <t>BN28NOVEMBER2026</t>
         </is>
       </c>
       <c r="C63" t="n">
@@ -1989,7 +1989,7 @@
       </c>
       <c r="E63" t="inlineStr">
         <is>
-          <t>https://raw.githubusercontent.com/DawSathaporn/BERNOVEM/main/BN24NOVEMBER2026</t>
+          <t>https://raw.githubusercontent.com/DawSathaporn/BERNOVEM/main/BN28NOVEMBER2026</t>
         </is>
       </c>
     </row>
@@ -2001,7 +2001,7 @@
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>BN25NOVEMBER2026</t>
+          <t>BN29NOVEMBER2026</t>
         </is>
       </c>
       <c r="C64" t="n">
@@ -2014,7 +2014,7 @@
       </c>
       <c r="E64" t="inlineStr">
         <is>
-          <t>https://raw.githubusercontent.com/DawSathaporn/BERNOVEM/main/BN25NOVEMBER2026</t>
+          <t>https://raw.githubusercontent.com/DawSathaporn/BERNOVEM/main/BN29NOVEMBER2026</t>
         </is>
       </c>
     </row>
@@ -2026,7 +2026,7 @@
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>BN26NOVEMBER2026</t>
+          <t>BN30NOVEMBER2026</t>
         </is>
       </c>
       <c r="C65" t="n">
@@ -2039,7 +2039,7 @@
       </c>
       <c r="E65" t="inlineStr">
         <is>
-          <t>https://raw.githubusercontent.com/DawSathaporn/BERNOVEM/main/BN26NOVEMBER2026</t>
+          <t>https://raw.githubusercontent.com/DawSathaporn/BERNOVEM/main/BN30NOVEMBER2026</t>
         </is>
       </c>
     </row>
@@ -2051,11 +2051,11 @@
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>BN27NOVEMBER2026</t>
+          <t>update_github_file.py</t>
         </is>
       </c>
       <c r="C66" t="n">
-        <v>889426</v>
+        <v>15175</v>
       </c>
       <c r="D66" t="inlineStr">
         <is>
@@ -2064,23 +2064,23 @@
       </c>
       <c r="E66" t="inlineStr">
         <is>
-          <t>https://raw.githubusercontent.com/DawSathaporn/BERNOVEM/main/BN27NOVEMBER2026</t>
+          <t>https://raw.githubusercontent.com/DawSathaporn/BERNOVEM/main/update_github_file.py</t>
         </is>
       </c>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>BERNOVEM</t>
+          <t>BEROKTO</t>
         </is>
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>BN28NOVEMBER2026</t>
+          <t>.github/workflows/main.yml</t>
         </is>
       </c>
       <c r="C67" t="n">
-        <v>889426</v>
+        <v>851</v>
       </c>
       <c r="D67" t="inlineStr">
         <is>
@@ -2089,23 +2089,23 @@
       </c>
       <c r="E67" t="inlineStr">
         <is>
-          <t>https://raw.githubusercontent.com/DawSathaporn/BERNOVEM/main/BN28NOVEMBER2026</t>
+          <t>https://raw.githubusercontent.com/DawSathaporn/BEROKTO/main/.github/workflows/main.yml</t>
         </is>
       </c>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>BERNOVEM</t>
+          <t>BEROKTO</t>
         </is>
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>BN29NOVEMBER2026</t>
+          <t>BR01OKTOBER2026</t>
         </is>
       </c>
       <c r="C68" t="n">
-        <v>889426</v>
+        <v>889425</v>
       </c>
       <c r="D68" t="inlineStr">
         <is>
@@ -2114,23 +2114,23 @@
       </c>
       <c r="E68" t="inlineStr">
         <is>
-          <t>https://raw.githubusercontent.com/DawSathaporn/BERNOVEM/main/BN29NOVEMBER2026</t>
+          <t>https://raw.githubusercontent.com/DawSathaporn/BEROKTO/main/BR01OKTOBER2026</t>
         </is>
       </c>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>BERNOVEM</t>
+          <t>BEROKTO</t>
         </is>
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>BN30NOVEMBER2026</t>
+          <t>BR02OKTOBER2026</t>
         </is>
       </c>
       <c r="C69" t="n">
-        <v>889426</v>
+        <v>889425</v>
       </c>
       <c r="D69" t="inlineStr">
         <is>
@@ -2139,23 +2139,23 @@
       </c>
       <c r="E69" t="inlineStr">
         <is>
-          <t>https://raw.githubusercontent.com/DawSathaporn/BERNOVEM/main/BN30NOVEMBER2026</t>
+          <t>https://raw.githubusercontent.com/DawSathaporn/BEROKTO/main/BR02OKTOBER2026</t>
         </is>
       </c>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>BERNOVEM</t>
+          <t>BEROKTO</t>
         </is>
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>update_github_file.py</t>
+          <t>BR03OKTOBER2026</t>
         </is>
       </c>
       <c r="C70" t="n">
-        <v>15175</v>
+        <v>889425</v>
       </c>
       <c r="D70" t="inlineStr">
         <is>
@@ -2164,23 +2164,23 @@
       </c>
       <c r="E70" t="inlineStr">
         <is>
-          <t>https://raw.githubusercontent.com/DawSathaporn/BERNOVEM/main/update_github_file.py</t>
+          <t>https://raw.githubusercontent.com/DawSathaporn/BEROKTO/main/BR03OKTOBER2026</t>
         </is>
       </c>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>BERDESEM</t>
+          <t>BEROKTO</t>
         </is>
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>.github/workflows/main.yml</t>
+          <t>BR04OKTOBER2026</t>
         </is>
       </c>
       <c r="C71" t="n">
-        <v>851</v>
+        <v>889425</v>
       </c>
       <c r="D71" t="inlineStr">
         <is>
@@ -2189,23 +2189,23 @@
       </c>
       <c r="E71" t="inlineStr">
         <is>
-          <t>https://raw.githubusercontent.com/DawSathaporn/BERDESEM/main/.github/workflows/main.yml</t>
+          <t>https://raw.githubusercontent.com/DawSathaporn/BEROKTO/main/BR04OKTOBER2026</t>
         </is>
       </c>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>BERDESEM</t>
+          <t>BEROKTO</t>
         </is>
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>BS01DESEMBER2026</t>
+          <t>BR05OKTOBER2026</t>
         </is>
       </c>
       <c r="C72" t="n">
-        <v>889426</v>
+        <v>889425</v>
       </c>
       <c r="D72" t="inlineStr">
         <is>
@@ -2214,23 +2214,23 @@
       </c>
       <c r="E72" t="inlineStr">
         <is>
-          <t>https://raw.githubusercontent.com/DawSathaporn/BERDESEM/main/BS01DESEMBER2026</t>
+          <t>https://raw.githubusercontent.com/DawSathaporn/BEROKTO/main/BR05OKTOBER2026</t>
         </is>
       </c>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>BERDESEM</t>
+          <t>BEROKTO</t>
         </is>
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>BS02DESEMBER2026</t>
+          <t>BR06OKTOBER2026</t>
         </is>
       </c>
       <c r="C73" t="n">
-        <v>889426</v>
+        <v>889425</v>
       </c>
       <c r="D73" t="inlineStr">
         <is>
@@ -2239,23 +2239,23 @@
       </c>
       <c r="E73" t="inlineStr">
         <is>
-          <t>https://raw.githubusercontent.com/DawSathaporn/BERDESEM/main/BS02DESEMBER2026</t>
+          <t>https://raw.githubusercontent.com/DawSathaporn/BEROKTO/main/BR06OKTOBER2026</t>
         </is>
       </c>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>BERDESEM</t>
+          <t>BEROKTO</t>
         </is>
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>BS03DESEMBER2026</t>
+          <t>BR07OKTOBER2026</t>
         </is>
       </c>
       <c r="C74" t="n">
-        <v>889426</v>
+        <v>889425</v>
       </c>
       <c r="D74" t="inlineStr">
         <is>
@@ -2264,23 +2264,23 @@
       </c>
       <c r="E74" t="inlineStr">
         <is>
-          <t>https://raw.githubusercontent.com/DawSathaporn/BERDESEM/main/BS03DESEMBER2026</t>
+          <t>https://raw.githubusercontent.com/DawSathaporn/BEROKTO/main/BR07OKTOBER2026</t>
         </is>
       </c>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>BERDESEM</t>
+          <t>BEROKTO</t>
         </is>
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>BS04DESEMBER2026</t>
+          <t>BR08OKTOBER2026</t>
         </is>
       </c>
       <c r="C75" t="n">
-        <v>889426</v>
+        <v>889425</v>
       </c>
       <c r="D75" t="inlineStr">
         <is>
@@ -2289,23 +2289,23 @@
       </c>
       <c r="E75" t="inlineStr">
         <is>
-          <t>https://raw.githubusercontent.com/DawSathaporn/BERDESEM/main/BS04DESEMBER2026</t>
+          <t>https://raw.githubusercontent.com/DawSathaporn/BEROKTO/main/BR08OKTOBER2026</t>
         </is>
       </c>
     </row>
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>BERDESEM</t>
+          <t>BEROKTO</t>
         </is>
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>BS05DESEMBER2026</t>
+          <t>BR09OKTOBER2026</t>
         </is>
       </c>
       <c r="C76" t="n">
-        <v>889426</v>
+        <v>889425</v>
       </c>
       <c r="D76" t="inlineStr">
         <is>
@@ -2314,23 +2314,23 @@
       </c>
       <c r="E76" t="inlineStr">
         <is>
-          <t>https://raw.githubusercontent.com/DawSathaporn/BERDESEM/main/BS05DESEMBER2026</t>
+          <t>https://raw.githubusercontent.com/DawSathaporn/BEROKTO/main/BR09OKTOBER2026</t>
         </is>
       </c>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>BERDESEM</t>
+          <t>BEROKTO</t>
         </is>
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>BS06DESEMBER2026</t>
+          <t>BR10OKTOBER2026</t>
         </is>
       </c>
       <c r="C77" t="n">
-        <v>889426</v>
+        <v>889425</v>
       </c>
       <c r="D77" t="inlineStr">
         <is>
@@ -2339,23 +2339,23 @@
       </c>
       <c r="E77" t="inlineStr">
         <is>
-          <t>https://raw.githubusercontent.com/DawSathaporn/BERDESEM/main/BS06DESEMBER2026</t>
+          <t>https://raw.githubusercontent.com/DawSathaporn/BEROKTO/main/BR10OKTOBER2026</t>
         </is>
       </c>
     </row>
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>BERDESEM</t>
+          <t>BEROKTO</t>
         </is>
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>BS07DESEMBER2026</t>
+          <t>BR11OKTOBER2026</t>
         </is>
       </c>
       <c r="C78" t="n">
-        <v>889426</v>
+        <v>889425</v>
       </c>
       <c r="D78" t="inlineStr">
         <is>
@@ -2364,23 +2364,23 @@
       </c>
       <c r="E78" t="inlineStr">
         <is>
-          <t>https://raw.githubusercontent.com/DawSathaporn/BERDESEM/main/BS07DESEMBER2026</t>
+          <t>https://raw.githubusercontent.com/DawSathaporn/BEROKTO/main/BR11OKTOBER2026</t>
         </is>
       </c>
     </row>
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>BERDESEM</t>
+          <t>BEROKTO</t>
         </is>
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>BS08DESEMBER2026</t>
+          <t>BR12OKTOBER2026</t>
         </is>
       </c>
       <c r="C79" t="n">
-        <v>889426</v>
+        <v>889425</v>
       </c>
       <c r="D79" t="inlineStr">
         <is>
@@ -2389,23 +2389,23 @@
       </c>
       <c r="E79" t="inlineStr">
         <is>
-          <t>https://raw.githubusercontent.com/DawSathaporn/BERDESEM/main/BS08DESEMBER2026</t>
+          <t>https://raw.githubusercontent.com/DawSathaporn/BEROKTO/main/BR12OKTOBER2026</t>
         </is>
       </c>
     </row>
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>BERDESEM</t>
+          <t>BEROKTO</t>
         </is>
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>BS09DESEMBER2026</t>
+          <t>BR13OKTOBER2026</t>
         </is>
       </c>
       <c r="C80" t="n">
-        <v>889426</v>
+        <v>889425</v>
       </c>
       <c r="D80" t="inlineStr">
         <is>
@@ -2414,23 +2414,23 @@
       </c>
       <c r="E80" t="inlineStr">
         <is>
-          <t>https://raw.githubusercontent.com/DawSathaporn/BERDESEM/main/BS09DESEMBER2026</t>
+          <t>https://raw.githubusercontent.com/DawSathaporn/BEROKTO/main/BR13OKTOBER2026</t>
         </is>
       </c>
     </row>
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>BERDESEM</t>
+          <t>BEROKTO</t>
         </is>
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>BS10DESEMBER2026</t>
+          <t>BR14OKTOBER2026</t>
         </is>
       </c>
       <c r="C81" t="n">
-        <v>889426</v>
+        <v>889425</v>
       </c>
       <c r="D81" t="inlineStr">
         <is>
@@ -2439,23 +2439,23 @@
       </c>
       <c r="E81" t="inlineStr">
         <is>
-          <t>https://raw.githubusercontent.com/DawSathaporn/BERDESEM/main/BS10DESEMBER2026</t>
+          <t>https://raw.githubusercontent.com/DawSathaporn/BEROKTO/main/BR14OKTOBER2026</t>
         </is>
       </c>
     </row>
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>BERDESEM</t>
+          <t>BEROKTO</t>
         </is>
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>BS11DESEMBER2026</t>
+          <t>BR15OKTOBER2026</t>
         </is>
       </c>
       <c r="C82" t="n">
-        <v>889426</v>
+        <v>889425</v>
       </c>
       <c r="D82" t="inlineStr">
         <is>
@@ -2464,23 +2464,23 @@
       </c>
       <c r="E82" t="inlineStr">
         <is>
-          <t>https://raw.githubusercontent.com/DawSathaporn/BERDESEM/main/BS11DESEMBER2026</t>
+          <t>https://raw.githubusercontent.com/DawSathaporn/BEROKTO/main/BR15OKTOBER2026</t>
         </is>
       </c>
     </row>
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>BERDESEM</t>
+          <t>BEROKTO</t>
         </is>
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>BS12DESEMBER2026</t>
+          <t>BR16OKTOBER2026</t>
         </is>
       </c>
       <c r="C83" t="n">
-        <v>889426</v>
+        <v>889425</v>
       </c>
       <c r="D83" t="inlineStr">
         <is>
@@ -2489,23 +2489,23 @@
       </c>
       <c r="E83" t="inlineStr">
         <is>
-          <t>https://raw.githubusercontent.com/DawSathaporn/BERDESEM/main/BS12DESEMBER2026</t>
+          <t>https://raw.githubusercontent.com/DawSathaporn/BEROKTO/main/BR16OKTOBER2026</t>
         </is>
       </c>
     </row>
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>BERDESEM</t>
+          <t>BEROKTO</t>
         </is>
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>BS13DESEMBER2026</t>
+          <t>BR17OKTOBER2026</t>
         </is>
       </c>
       <c r="C84" t="n">
-        <v>889426</v>
+        <v>889425</v>
       </c>
       <c r="D84" t="inlineStr">
         <is>
@@ -2514,23 +2514,23 @@
       </c>
       <c r="E84" t="inlineStr">
         <is>
-          <t>https://raw.githubusercontent.com/DawSathaporn/BERDESEM/main/BS13DESEMBER2026</t>
+          <t>https://raw.githubusercontent.com/DawSathaporn/BEROKTO/main/BR17OKTOBER2026</t>
         </is>
       </c>
     </row>
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>BERDESEM</t>
+          <t>BEROKTO</t>
         </is>
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>BS14DESEMBER2026</t>
+          <t>BR18OKTOBER2026</t>
         </is>
       </c>
       <c r="C85" t="n">
-        <v>889426</v>
+        <v>889425</v>
       </c>
       <c r="D85" t="inlineStr">
         <is>
@@ -2539,23 +2539,23 @@
       </c>
       <c r="E85" t="inlineStr">
         <is>
-          <t>https://raw.githubusercontent.com/DawSathaporn/BERDESEM/main/BS14DESEMBER2026</t>
+          <t>https://raw.githubusercontent.com/DawSathaporn/BEROKTO/main/BR18OKTOBER2026</t>
         </is>
       </c>
     </row>
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>BERDESEM</t>
+          <t>BEROKTO</t>
         </is>
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>BS15DESEMBER2026</t>
+          <t>BR19OKTOBER2026</t>
         </is>
       </c>
       <c r="C86" t="n">
-        <v>889426</v>
+        <v>889425</v>
       </c>
       <c r="D86" t="inlineStr">
         <is>
@@ -2564,23 +2564,23 @@
       </c>
       <c r="E86" t="inlineStr">
         <is>
-          <t>https://raw.githubusercontent.com/DawSathaporn/BERDESEM/main/BS15DESEMBER2026</t>
+          <t>https://raw.githubusercontent.com/DawSathaporn/BEROKTO/main/BR19OKTOBER2026</t>
         </is>
       </c>
     </row>
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>BERDESEM</t>
+          <t>BEROKTO</t>
         </is>
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>BS16DESEMBER2026</t>
+          <t>BR20OKTOBER2026</t>
         </is>
       </c>
       <c r="C87" t="n">
-        <v>889426</v>
+        <v>889425</v>
       </c>
       <c r="D87" t="inlineStr">
         <is>
@@ -2589,23 +2589,23 @@
       </c>
       <c r="E87" t="inlineStr">
         <is>
-          <t>https://raw.githubusercontent.com/DawSathaporn/BERDESEM/main/BS16DESEMBER2026</t>
+          <t>https://raw.githubusercontent.com/DawSathaporn/BEROKTO/main/BR20OKTOBER2026</t>
         </is>
       </c>
     </row>
     <row r="88">
       <c r="A88" t="inlineStr">
         <is>
-          <t>BERDESEM</t>
+          <t>BEROKTO</t>
         </is>
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>BS17DESEMBER2026</t>
+          <t>BR21OKTOBER2026</t>
         </is>
       </c>
       <c r="C88" t="n">
-        <v>889426</v>
+        <v>889425</v>
       </c>
       <c r="D88" t="inlineStr">
         <is>
@@ -2614,23 +2614,23 @@
       </c>
       <c r="E88" t="inlineStr">
         <is>
-          <t>https://raw.githubusercontent.com/DawSathaporn/BERDESEM/main/BS17DESEMBER2026</t>
+          <t>https://raw.githubusercontent.com/DawSathaporn/BEROKTO/main/BR21OKTOBER2026</t>
         </is>
       </c>
     </row>
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>BERDESEM</t>
+          <t>BEROKTO</t>
         </is>
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t>BS18DESEMBER2026</t>
+          <t>BR22OKTOBER2026</t>
         </is>
       </c>
       <c r="C89" t="n">
-        <v>889426</v>
+        <v>889425</v>
       </c>
       <c r="D89" t="inlineStr">
         <is>
@@ -2639,23 +2639,23 @@
       </c>
       <c r="E89" t="inlineStr">
         <is>
-          <t>https://raw.githubusercontent.com/DawSathaporn/BERDESEM/main/BS18DESEMBER2026</t>
+          <t>https://raw.githubusercontent.com/DawSathaporn/BEROKTO/main/BR22OKTOBER2026</t>
         </is>
       </c>
     </row>
     <row r="90">
       <c r="A90" t="inlineStr">
         <is>
-          <t>BERDESEM</t>
+          <t>BEROKTO</t>
         </is>
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t>BS19DESEMBER2026</t>
+          <t>BR23OKTOBER2026</t>
         </is>
       </c>
       <c r="C90" t="n">
-        <v>889426</v>
+        <v>889425</v>
       </c>
       <c r="D90" t="inlineStr">
         <is>
@@ -2664,23 +2664,23 @@
       </c>
       <c r="E90" t="inlineStr">
         <is>
-          <t>https://raw.githubusercontent.com/DawSathaporn/BERDESEM/main/BS19DESEMBER2026</t>
+          <t>https://raw.githubusercontent.com/DawSathaporn/BEROKTO/main/BR23OKTOBER2026</t>
         </is>
       </c>
     </row>
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>BERDESEM</t>
+          <t>BEROKTO</t>
         </is>
       </c>
       <c r="B91" t="inlineStr">
         <is>
-          <t>BS20DESEMBER2026</t>
+          <t>BR24OKTOBER2026</t>
         </is>
       </c>
       <c r="C91" t="n">
-        <v>889426</v>
+        <v>889425</v>
       </c>
       <c r="D91" t="inlineStr">
         <is>
@@ -2689,23 +2689,23 @@
       </c>
       <c r="E91" t="inlineStr">
         <is>
-          <t>https://raw.githubusercontent.com/DawSathaporn/BERDESEM/main/BS20DESEMBER2026</t>
+          <t>https://raw.githubusercontent.com/DawSathaporn/BEROKTO/main/BR24OKTOBER2026</t>
         </is>
       </c>
     </row>
     <row r="92">
       <c r="A92" t="inlineStr">
         <is>
-          <t>BERDESEM</t>
+          <t>BEROKTO</t>
         </is>
       </c>
       <c r="B92" t="inlineStr">
         <is>
-          <t>BS21DESEMBER2026</t>
+          <t>BR25OKTOBER2026</t>
         </is>
       </c>
       <c r="C92" t="n">
-        <v>889426</v>
+        <v>889425</v>
       </c>
       <c r="D92" t="inlineStr">
         <is>
@@ -2714,23 +2714,23 @@
       </c>
       <c r="E92" t="inlineStr">
         <is>
-          <t>https://raw.githubusercontent.com/DawSathaporn/BERDESEM/main/BS21DESEMBER2026</t>
+          <t>https://raw.githubusercontent.com/DawSathaporn/BEROKTO/main/BR25OKTOBER2026</t>
         </is>
       </c>
     </row>
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>BERDESEM</t>
+          <t>BEROKTO</t>
         </is>
       </c>
       <c r="B93" t="inlineStr">
         <is>
-          <t>BS22DESEMBER2026</t>
+          <t>BR26OKTOBER2026</t>
         </is>
       </c>
       <c r="C93" t="n">
-        <v>889426</v>
+        <v>889425</v>
       </c>
       <c r="D93" t="inlineStr">
         <is>
@@ -2739,23 +2739,23 @@
       </c>
       <c r="E93" t="inlineStr">
         <is>
-          <t>https://raw.githubusercontent.com/DawSathaporn/BERDESEM/main/BS22DESEMBER2026</t>
+          <t>https://raw.githubusercontent.com/DawSathaporn/BEROKTO/main/BR26OKTOBER2026</t>
         </is>
       </c>
     </row>
     <row r="94">
       <c r="A94" t="inlineStr">
         <is>
-          <t>BERDESEM</t>
+          <t>BEROKTO</t>
         </is>
       </c>
       <c r="B94" t="inlineStr">
         <is>
-          <t>BS23DESEMBER2026</t>
+          <t>BR27OKTOBER2026</t>
         </is>
       </c>
       <c r="C94" t="n">
-        <v>889426</v>
+        <v>889425</v>
       </c>
       <c r="D94" t="inlineStr">
         <is>
@@ -2764,23 +2764,23 @@
       </c>
       <c r="E94" t="inlineStr">
         <is>
-          <t>https://raw.githubusercontent.com/DawSathaporn/BERDESEM/main/BS23DESEMBER2026</t>
+          <t>https://raw.githubusercontent.com/DawSathaporn/BEROKTO/main/BR27OKTOBER2026</t>
         </is>
       </c>
     </row>
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>BERDESEM</t>
+          <t>BEROKTO</t>
         </is>
       </c>
       <c r="B95" t="inlineStr">
         <is>
-          <t>BS24DESEMBER2026</t>
+          <t>BR28OKTOBER2026</t>
         </is>
       </c>
       <c r="C95" t="n">
-        <v>889426</v>
+        <v>889425</v>
       </c>
       <c r="D95" t="inlineStr">
         <is>
@@ -2789,23 +2789,23 @@
       </c>
       <c r="E95" t="inlineStr">
         <is>
-          <t>https://raw.githubusercontent.com/DawSathaporn/BERDESEM/main/BS24DESEMBER2026</t>
+          <t>https://raw.githubusercontent.com/DawSathaporn/BEROKTO/main/BR28OKTOBER2026</t>
         </is>
       </c>
     </row>
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
-          <t>BERDESEM</t>
+          <t>BEROKTO</t>
         </is>
       </c>
       <c r="B96" t="inlineStr">
         <is>
-          <t>BS25DESEMBER2026</t>
+          <t>BR29OKTOBER2026</t>
         </is>
       </c>
       <c r="C96" t="n">
-        <v>889426</v>
+        <v>889425</v>
       </c>
       <c r="D96" t="inlineStr">
         <is>
@@ -2814,23 +2814,23 @@
       </c>
       <c r="E96" t="inlineStr">
         <is>
-          <t>https://raw.githubusercontent.com/DawSathaporn/BERDESEM/main/BS25DESEMBER2026</t>
+          <t>https://raw.githubusercontent.com/DawSathaporn/BEROKTO/main/BR29OKTOBER2026</t>
         </is>
       </c>
     </row>
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>BERDESEM</t>
+          <t>BEROKTO</t>
         </is>
       </c>
       <c r="B97" t="inlineStr">
         <is>
-          <t>BS26DESEMBER2026</t>
+          <t>BR30OKTOBER2026</t>
         </is>
       </c>
       <c r="C97" t="n">
-        <v>889426</v>
+        <v>889425</v>
       </c>
       <c r="D97" t="inlineStr">
         <is>
@@ -2839,23 +2839,23 @@
       </c>
       <c r="E97" t="inlineStr">
         <is>
-          <t>https://raw.githubusercontent.com/DawSathaporn/BERDESEM/main/BS26DESEMBER2026</t>
+          <t>https://raw.githubusercontent.com/DawSathaporn/BEROKTO/main/BR30OKTOBER2026</t>
         </is>
       </c>
     </row>
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t>BERDESEM</t>
+          <t>BEROKTO</t>
         </is>
       </c>
       <c r="B98" t="inlineStr">
         <is>
-          <t>BS27DESEMBER2026</t>
+          <t>BR31OKTOBER2026</t>
         </is>
       </c>
       <c r="C98" t="n">
-        <v>889426</v>
+        <v>889425</v>
       </c>
       <c r="D98" t="inlineStr">
         <is>
@@ -2864,23 +2864,23 @@
       </c>
       <c r="E98" t="inlineStr">
         <is>
-          <t>https://raw.githubusercontent.com/DawSathaporn/BERDESEM/main/BS27DESEMBER2026</t>
+          <t>https://raw.githubusercontent.com/DawSathaporn/BEROKTO/main/BR31OKTOBER2026</t>
         </is>
       </c>
     </row>
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>BERDESEM</t>
+          <t>BEROKTO</t>
         </is>
       </c>
       <c r="B99" t="inlineStr">
         <is>
-          <t>BS28DESEMBER2026</t>
+          <t>update_github_file.py</t>
         </is>
       </c>
       <c r="C99" t="n">
-        <v>889426</v>
+        <v>15172</v>
       </c>
       <c r="D99" t="inlineStr">
         <is>
@@ -2889,23 +2889,23 @@
       </c>
       <c r="E99" t="inlineStr">
         <is>
-          <t>https://raw.githubusercontent.com/DawSathaporn/BERDESEM/main/BS28DESEMBER2026</t>
+          <t>https://raw.githubusercontent.com/DawSathaporn/BEROKTO/main/update_github_file.py</t>
         </is>
       </c>
     </row>
     <row r="100">
       <c r="A100" t="inlineStr">
         <is>
-          <t>BERDESEM</t>
+          <t>UGR</t>
         </is>
       </c>
       <c r="B100" t="inlineStr">
         <is>
-          <t>BS29DESEMBER2026</t>
+          <t>.github/workflows/raw-urls.yml</t>
         </is>
       </c>
       <c r="C100" t="n">
-        <v>889426</v>
+        <v>2174</v>
       </c>
       <c r="D100" t="inlineStr">
         <is>
@@ -2914,23 +2914,23 @@
       </c>
       <c r="E100" t="inlineStr">
         <is>
-          <t>https://raw.githubusercontent.com/DawSathaporn/BERDESEM/main/BS29DESEMBER2026</t>
+          <t>https://raw.githubusercontent.com/DawSathaporn/UGR/main/.github/workflows/raw-urls.yml</t>
         </is>
       </c>
     </row>
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>BERDESEM</t>
+          <t>UGR</t>
         </is>
       </c>
       <c r="B101" t="inlineStr">
         <is>
-          <t>BS30DESEMBER2026</t>
+          <t>data/DawSathaporn_all_raw.csv</t>
         </is>
       </c>
       <c r="C101" t="n">
-        <v>889426</v>
+        <v>11875</v>
       </c>
       <c r="D101" t="inlineStr">
         <is>
@@ -2939,23 +2939,23 @@
       </c>
       <c r="E101" t="inlineStr">
         <is>
-          <t>https://raw.githubusercontent.com/DawSathaporn/BERDESEM/main/BS30DESEMBER2026</t>
+          <t>https://raw.githubusercontent.com/DawSathaporn/UGR/main/data/DawSathaporn_all_raw.csv</t>
         </is>
       </c>
     </row>
     <row r="102">
       <c r="A102" t="inlineStr">
         <is>
-          <t>BERDESEM</t>
+          <t>UGR</t>
         </is>
       </c>
       <c r="B102" t="inlineStr">
         <is>
-          <t>BS31DESEMBER2026</t>
+          <t>data/DawSathaporn_all_raw.xlsx</t>
         </is>
       </c>
       <c r="C102" t="n">
-        <v>889426</v>
+        <v>7706</v>
       </c>
       <c r="D102" t="inlineStr">
         <is>
@@ -2964,23 +2964,23 @@
       </c>
       <c r="E102" t="inlineStr">
         <is>
-          <t>https://raw.githubusercontent.com/DawSathaporn/BERDESEM/main/BS31DESEMBER2026</t>
+          <t>https://raw.githubusercontent.com/DawSathaporn/UGR/main/data/DawSathaporn_all_raw.xlsx</t>
         </is>
       </c>
     </row>
     <row r="103">
       <c r="A103" t="inlineStr">
         <is>
-          <t>BERDESEM</t>
+          <t>UGR</t>
         </is>
       </c>
       <c r="B103" t="inlineStr">
         <is>
-          <t>update_github_file.py</t>
+          <t>data/uppermoon77_all_raw.csv</t>
         </is>
       </c>
       <c r="C103" t="n">
-        <v>15175</v>
+        <v>41907</v>
       </c>
       <c r="D103" t="inlineStr">
         <is>
@@ -2989,7 +2989,57 @@
       </c>
       <c r="E103" t="inlineStr">
         <is>
-          <t>https://raw.githubusercontent.com/DawSathaporn/BERDESEM/main/update_github_file.py</t>
+          <t>https://raw.githubusercontent.com/DawSathaporn/UGR/main/data/uppermoon77_all_raw.csv</t>
+        </is>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" t="inlineStr">
+        <is>
+          <t>UGR</t>
+        </is>
+      </c>
+      <c r="B104" t="inlineStr">
+        <is>
+          <t>data/uppermoon77_all_raw.xlsx</t>
+        </is>
+      </c>
+      <c r="C104" t="n">
+        <v>15208</v>
+      </c>
+      <c r="D104" t="inlineStr">
+        <is>
+          <t>main</t>
+        </is>
+      </c>
+      <c r="E104" t="inlineStr">
+        <is>
+          <t>https://raw.githubusercontent.com/DawSathaporn/UGR/main/data/uppermoon77_all_raw.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" t="inlineStr">
+        <is>
+          <t>UGR</t>
+        </is>
+      </c>
+      <c r="B105" t="inlineStr">
+        <is>
+          <t>generate_all_repos_raw_urls.py</t>
+        </is>
+      </c>
+      <c r="C105" t="n">
+        <v>6543</v>
+      </c>
+      <c r="D105" t="inlineStr">
+        <is>
+          <t>main</t>
+        </is>
+      </c>
+      <c r="E105" t="inlineStr">
+        <is>
+          <t>https://raw.githubusercontent.com/DawSathaporn/UGR/main/generate_all_repos_raw_urls.py</t>
         </is>
       </c>
     </row>

</xml_diff>